<commit_message>
cluster analysis of factoriescap_s costs 0
</commit_message>
<xml_diff>
--- a/clustering/Clusters 4 factoriescap_s (costs) 0.xlsx
+++ b/clustering/Clusters 4 factoriescap_s (costs) 0.xlsx
@@ -529,6 +529,8 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
   </fonts>
   <fills count="2">
@@ -879,11 +881,7 @@
   <dimension ref="A1:H232"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="73.5703125" customWidth="1"/>
-    <col min="4" max="4" width="17.140625" customWidth="1"/>
-    <col min="5" max="5" width="16.28515625" customWidth="1"/>
-    <col min="6" max="6" width="15.7109375" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="1" max="1" width="82" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6712,25 +6710,25 @@
     </row>
     <row r="225" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A225" s="2" t="s">
-        <v>162</v>
+        <v>140</v>
       </c>
       <c r="B225" s="2" t="s">
-        <v>163</v>
+        <v>141</v>
       </c>
       <c r="C225" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="D225" s="2">
-        <v>74573767</v>
+        <v>13477792</v>
       </c>
       <c r="E225" s="2">
-        <v>212048.78478367999</v>
+        <v>28777.807271819998</v>
       </c>
       <c r="F225" s="2">
-        <v>7049.4571275200014</v>
+        <v>5240.6774820000001</v>
       </c>
       <c r="G225" s="2">
-        <v>281.43069239999983</v>
+        <v>6.7763591199995874</v>
       </c>
       <c r="H225" s="2">
         <v>1</v>
@@ -6738,51 +6736,51 @@
     </row>
     <row r="226" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A226" s="2" t="s">
-        <v>140</v>
+        <v>58</v>
       </c>
       <c r="B226" s="2" t="s">
-        <v>141</v>
+        <v>59</v>
       </c>
       <c r="C226" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="D226" s="2">
-        <v>13477792</v>
+        <v>23598403</v>
       </c>
       <c r="E226" s="2">
-        <v>28777.807271819998</v>
+        <v>61599.78433853999</v>
       </c>
       <c r="F226" s="2">
-        <v>5240.6774820000001</v>
+        <v>1184.0482836000001</v>
       </c>
       <c r="G226" s="2">
-        <v>6.7763591199995874</v>
+        <v>6438.3812715599997</v>
       </c>
       <c r="H226" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="227" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A227" s="2" t="s">
-        <v>162</v>
+        <v>114</v>
       </c>
       <c r="B227" s="2" t="s">
-        <v>163</v>
+        <v>115</v>
       </c>
       <c r="C227" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="D227" s="2">
-        <v>66796992</v>
+        <v>723904.99999999453</v>
       </c>
       <c r="E227" s="2">
-        <v>258750.9908536</v>
+        <v>9537.5395684799951</v>
       </c>
       <c r="F227" s="2">
-        <v>6498.3629939000011</v>
+        <v>0.21320964000000001</v>
       </c>
       <c r="G227" s="2">
-        <v>985.79842147999943</v>
+        <v>6388.6231835999988</v>
       </c>
       <c r="H227" s="2">
         <v>2</v>
@@ -6796,22 +6794,22 @@
         <v>163</v>
       </c>
       <c r="C228" s="2">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="D228" s="2">
-        <v>62978040</v>
+        <v>74573767</v>
       </c>
       <c r="E228" s="2">
-        <v>235445.33845601999</v>
+        <v>212048.78478367999</v>
       </c>
       <c r="F228" s="2">
-        <v>978.37784099999919</v>
+        <v>7049.4571275200014</v>
       </c>
       <c r="G228" s="2">
-        <v>676.24855955999988</v>
+        <v>281.43069239999983</v>
       </c>
       <c r="H228" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="229" spans="1:8" x14ac:dyDescent="0.25">
@@ -6822,22 +6820,22 @@
         <v>163</v>
       </c>
       <c r="C229" s="2">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="D229" s="2">
-        <v>50017917.000000007</v>
+        <v>66796992</v>
       </c>
       <c r="E229" s="2">
-        <v>193299.219548875</v>
+        <v>258750.9908536</v>
       </c>
       <c r="F229" s="2">
-        <v>1131.9292105</v>
+        <v>6498.3629939000011</v>
       </c>
       <c r="G229" s="2">
-        <v>1170.684354949999</v>
+        <v>985.79842147999943</v>
       </c>
       <c r="H229" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="230" spans="1:8" x14ac:dyDescent="0.25">
@@ -6848,45 +6846,45 @@
         <v>163</v>
       </c>
       <c r="C230" s="2">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="D230" s="2">
-        <v>87323581</v>
+        <v>62978040</v>
       </c>
       <c r="E230" s="2">
-        <v>220411.94692799999</v>
+        <v>235445.33845601999</v>
       </c>
       <c r="F230" s="2">
-        <v>1905.2652479999999</v>
+        <v>978.37784099999919</v>
       </c>
       <c r="G230" s="2">
-        <v>768.4297439999998</v>
+        <v>676.24855955999988</v>
       </c>
       <c r="H230" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="231" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A231" s="2" t="s">
-        <v>58</v>
+        <v>162</v>
       </c>
       <c r="B231" s="2" t="s">
-        <v>59</v>
+        <v>163</v>
       </c>
       <c r="C231" s="2">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="D231" s="2">
-        <v>23598403</v>
+        <v>50017917.000000007</v>
       </c>
       <c r="E231" s="2">
-        <v>61599.78433853999</v>
+        <v>193299.219548875</v>
       </c>
       <c r="F231" s="2">
-        <v>1184.0482836000001</v>
+        <v>1131.9292105</v>
       </c>
       <c r="G231" s="2">
-        <v>6438.3812715599997</v>
+        <v>1170.684354949999</v>
       </c>
       <c r="H231" s="2">
         <v>3</v>
@@ -6894,25 +6892,25 @@
     </row>
     <row r="232" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A232" s="2" t="s">
-        <v>114</v>
+        <v>162</v>
       </c>
       <c r="B232" s="2" t="s">
-        <v>115</v>
+        <v>163</v>
       </c>
       <c r="C232" s="2">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="D232" s="2">
-        <v>723904.99999999453</v>
+        <v>87323581</v>
       </c>
       <c r="E232" s="2">
-        <v>9537.5395684799951</v>
+        <v>220411.94692799999</v>
       </c>
       <c r="F232" s="2">
-        <v>0.21320964000000001</v>
+        <v>1905.2652479999999</v>
       </c>
       <c r="G232" s="2">
-        <v>6388.6231835999988</v>
+        <v>768.4297439999998</v>
       </c>
       <c r="H232" s="2">
         <v>3</v>

</xml_diff>